<commit_message>
docs & templates: sanitize master budget template and update guides
- Completely scrub personal PII, specific team names, account numbers, and historical balances from master budget template
- Update master template with generic placeholders while preserving all dynamic formula links
- Update live Google Sheet template in-place (ID: 1W6-_pH7H24ogvHRtxeRjiNFfoL9HHKs6ZtIjBTk_4Z4)
- Sanitize sponsorship workflow guide and Apps Script template with configurable variables
- Add HCR volunteer onboarding guide and step-by-step UI references
- Add google-drive-staging/ to .gitignore
</commit_message>
<xml_diff>
--- a/templates/TAMHA_Team_Budget_Master_Template.xlsx
+++ b/templates/TAMHA_Team_Budget_Master_Template.xlsx
@@ -634,9 +634,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
@@ -664,7 +664,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Truro Bearcats U13 A</t>
+          <t>[Enter Team Name - e.g., Truro Bearcats U13 A]</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Tom Malone</t>
+          <t>[Head Coach Full Name]</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Matt Redmond</t>
+          <t>[Team Manager Full Name]</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -714,7 +714,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Amy Redmond</t>
+          <t>[Team Treasurer Full Name]</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>299688400</t>
+          <t>[Enter 9-Digit Account #]</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Initial Budget (Oct 30)</t>
+          <t>Preliminary Budget (Oct 30)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1632,7 +1632,7 @@
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
         <is>
-          <t>Major Corporate Sponsor (e.g. Jersey / Gold)</t>
+          <t>[Major Team Sponsor - e.g. Local Business]</t>
         </is>
       </c>
       <c r="B6" s="13" t="inlineStr">
@@ -1642,30 +1642,30 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Local Business Owner</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>E-transfer</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
         <v>1000</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 1 (Gold)</t>
+          <t>[Gold Banner Sponsor 1]</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
@@ -1675,30 +1675,30 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Cheque</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E7" s="11" t="n">
         <v>500</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 2 (Gold)</t>
+          <t>[Gold Banner Sponsor 2]</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
@@ -1708,30 +1708,30 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Cheque</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E8" s="11" t="n">
         <v>500</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 3 (Silver)</t>
+          <t>[Silver Banner Sponsor 1]</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
@@ -1741,30 +1741,30 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Cheque</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
         <v>250</v>
       </c>
       <c r="F9" s="11" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 4 (Silver)</t>
+          <t>[Silver Banner Sponsor 2]</t>
         </is>
       </c>
       <c r="B10" s="13" t="inlineStr">
@@ -1774,30 +1774,30 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>E-transfer</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
         <v>250</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 5 (Silver)</t>
+          <t>[Silver Banner Sponsor 3]</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
@@ -1807,30 +1807,30 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Cheque</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
         <v>250</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>250</v>
+        <v>0</v>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 6 (Bronze)</t>
+          <t>[Bronze Banner Sponsor 1]</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
@@ -1840,30 +1840,30 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
         <v>100</v>
       </c>
       <c r="F12" s="11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Banner Sponsor 7 (Bronze)</t>
+          <t>[Bronze Banner Sponsor 2]</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
@@ -1873,23 +1873,23 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Business Contact</t>
+          <t>[Contact Name]</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>E-transfer</t>
+          <t>[Cheque / E-transfer]</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
         <v>100</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
@@ -1959,24 +1959,24 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Team Bottle Drive (Fall)</t>
+          <t>[Team Bottle Drive - Fall]</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>Oct 19, 2026</t>
+          <t>[Oct 2026]</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Parent Volunteer</t>
+          <t>[Parent Volunteer]</t>
         </is>
       </c>
       <c r="D18" s="11" t="n">
-        <v>1200</v>
+        <v>1000</v>
       </c>
       <c r="E18" s="11" t="n">
-        <v>1368</v>
+        <v>0</v>
       </c>
       <c r="F18" s="11">
         <f>E18-D18</f>
@@ -1984,31 +1984,31 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Completed - Deposited</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Pot O' Gold 50/50 Raffle</t>
+          <t>[50/50 Raffle - e.g. Pot O' Gold]</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>Nov 15, 2026</t>
+          <t>[Nov 2026]</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>Treasurer</t>
+          <t>[Treasurer]</t>
         </is>
       </c>
       <c r="D19" s="11" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>1160</v>
+        <v>0</v>
       </c>
       <c r="F19" s="11">
         <f>E19-D19</f>
@@ -2016,31 +2016,31 @@
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>Completed - Net after prize</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Grand In Your Hand / Cash Draw</t>
+          <t>[Ticket Draw / Grand In Your Hand]</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Dec 10, 2026</t>
+          <t>[Dec 2026]</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>Team Manager</t>
+          <t>[Manager]</t>
         </is>
       </c>
       <c r="D20" s="11" t="n">
         <v>1000</v>
       </c>
       <c r="E20" s="11" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="F20" s="11">
         <f>E20-D20</f>
@@ -2048,28 +2048,28 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Super Bowl Square Board / Silent Auction</t>
+          <t>[Square Board / Silent Auction]</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Feb 7, 2027</t>
+          <t>[Feb 2027]</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>Parent Committee</t>
+          <t>[Parent Committee]</t>
         </is>
       </c>
       <c r="D21" s="11" t="n">
-        <v>800</v>
+        <v>500</v>
       </c>
       <c r="E21" s="11" t="n">
         <v>0</v>
@@ -2080,24 +2080,24 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>Planned for Winter</t>
+          <t>Planned</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Optional Team Fundraiser 5</t>
+          <t>[Optional Fundraiser 5]</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>[TBD]</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>Volunteer</t>
+          <t>[Volunteer]</t>
         </is>
       </c>
       <c r="D22" s="11" t="n">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Contingency</t>
+          <t>Optional</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
         <v/>
       </c>
       <c r="E27" s="11" t="n">
-        <v>3850</v>
+        <v>0</v>
       </c>
       <c r="F27" s="11">
         <f>E27-D27</f>
@@ -2230,7 +2230,7 @@
         <v/>
       </c>
       <c r="E28" s="11" t="n">
-        <v>3850</v>
+        <v>0</v>
       </c>
       <c r="F28" s="11">
         <f>E28-D28</f>
@@ -2260,7 +2260,7 @@
         <v/>
       </c>
       <c r="E29" s="11" t="n">
-        <v>1700</v>
+        <v>0</v>
       </c>
       <c r="F29" s="11">
         <f>E29-D29</f>
@@ -2386,7 +2386,7 @@
         <v/>
       </c>
       <c r="E37" s="11" t="n">
-        <v>2550</v>
+        <v>0</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -2519,7 +2519,7 @@
         <v/>
       </c>
       <c r="G49" s="28">
-        <f>IF(F49&gt;=0,"Surplus / Target Met","Deficit")</f>
+        <f>IF(F49&gt;=0,"Surplus / Target Met","Pending")</f>
         <v/>
       </c>
     </row>
@@ -2639,7 +2639,7 @@
         <v>3850</v>
       </c>
       <c r="F6" s="11" t="n">
-        <v>3850</v>
+        <v>0</v>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
@@ -2672,7 +2672,7 @@
         <v>3850</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>3850</v>
+        <v>0</v>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
@@ -2705,7 +2705,7 @@
         <v>550</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
@@ -2768,10 +2768,10 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="F10" s="11" t="n">
-        <v>1032.29</v>
+        <v>0</v>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
@@ -2848,7 +2848,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>Tournament 1: Early Bird / Challenge Cup</t>
+          <t>Tournament 1: [Early Bird / Pre-Season Event]</t>
         </is>
       </c>
       <c r="B18" s="13" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>Amherst, NS</t>
+          <t>[Host Town, NS]</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -2870,7 +2870,7 @@
         <v>850</v>
       </c>
       <c r="F18" s="11" t="n">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
@@ -2881,7 +2881,7 @@
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>Tournament 2: Holiday / New Year Invitational</t>
+          <t>Tournament 2: [Holiday / Winter Invitational]</t>
         </is>
       </c>
       <c r="B19" s="13" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>Local / Regional</t>
+          <t>[Host Town, NS]</t>
         </is>
       </c>
       <c r="D19" s="13" t="inlineStr">
@@ -2903,7 +2903,7 @@
         <v>900</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>867</v>
+        <v>0</v>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
@@ -2914,7 +2914,7 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Tournament 3: SEDMHA Tournament</t>
+          <t>Tournament 3: [SEDMHA / March Tournament]</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
@@ -2933,10 +2933,10 @@
         </is>
       </c>
       <c r="E20" s="11" t="n">
-        <v>1325</v>
+        <v>1200</v>
       </c>
       <c r="F20" s="11" t="n">
-        <v>1325</v>
+        <v>0</v>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
@@ -2947,7 +2947,7 @@
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>Tournament 4: Away / Friendship Tournament</t>
+          <t>Tournament 4: [Away / Travel Tournament]</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
@@ -2957,7 +2957,7 @@
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>PEI / New Brunswick</t>
+          <t>[PEI / NB / Local]</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -2969,7 +2969,7 @@
         <v>850</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
@@ -3056,23 +3056,23 @@
       </c>
       <c r="C28" s="13" t="inlineStr">
         <is>
-          <t>RECC / West Colchester</t>
+          <t>Local Rink / RECC</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Pre-Season / Mid-Season</t>
+          <t>Pre-Season / Practice</t>
         </is>
       </c>
       <c r="E28" s="11" t="n">
         <v>990</v>
       </c>
       <c r="F28" s="11" t="n">
-        <v>990</v>
+        <v>0</v>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>Extra development sessions</t>
+          <t>Extra team development ice</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="C29" s="13" t="inlineStr">
         <is>
-          <t>RECC Truro</t>
+          <t>Home Rink</t>
         </is>
       </c>
       <c r="D29" s="13" t="inlineStr">
@@ -3101,11 +3101,11 @@
         <v>516</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>516</v>
+        <v>0</v>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>Home exhibition games</t>
+          <t>Home exhibition game slots</t>
         </is>
       </c>
     </row>
@@ -3134,11 +3134,11 @@
         <v>180</v>
       </c>
       <c r="F30" s="11" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>2 refs + linesmen</t>
+          <t>Cash payout for officials</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="C31" s="13" t="inlineStr">
         <is>
-          <t>Truro Timekeepers</t>
+          <t>Timekeeper Association</t>
         </is>
       </c>
       <c r="D31" s="13" t="inlineStr">
@@ -3167,11 +3167,11 @@
         <v>60</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Electronic game sheet / clock</t>
+          <t>Clock / game sheet operator</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
         <v>550</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="G37" s="10" t="inlineStr">
         <is>
@@ -3282,7 +3282,7 @@
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Retractable / Arena Banner</t>
+          <t>Arena Display Banner</t>
         </is>
       </c>
       <c r="C38" s="13" t="inlineStr">
@@ -3299,7 +3299,7 @@
         <v>200</v>
       </c>
       <c r="F38" s="11" t="n">
-        <v>168.59</v>
+        <v>0</v>
       </c>
       <c r="G38" s="10" t="inlineStr">
         <is>
@@ -3332,7 +3332,7 @@
         <v>250</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>245.59</v>
+        <v>0</v>
       </c>
       <c r="G39" s="10" t="inlineStr">
         <is>
@@ -3365,7 +3365,7 @@
         <v>680</v>
       </c>
       <c r="F40" s="11" t="n">
-        <v>680</v>
+        <v>0</v>
       </c>
       <c r="G40" s="10" t="inlineStr">
         <is>
@@ -3398,7 +3398,7 @@
         <v>100</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="G41" s="10" t="inlineStr">
         <is>
@@ -3431,11 +3431,11 @@
         <v>120</v>
       </c>
       <c r="F42" s="11" t="n">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="G42" s="10" t="inlineStr">
         <is>
-          <t>Team equipment</t>
+          <t>Team practice equipment</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
         <v>450</v>
       </c>
       <c r="F47" s="11" t="n">
-        <v>473.51</v>
+        <v>0</v>
       </c>
       <c r="G47" s="10" t="inlineStr">
         <is>
@@ -3563,7 +3563,7 @@
         <v>500</v>
       </c>
       <c r="F48" s="11" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="G48" s="10" t="inlineStr">
         <is>
@@ -3596,7 +3596,7 @@
         <v>250</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>282.85</v>
+        <v>0</v>
       </c>
       <c r="G49" s="10" t="inlineStr">
         <is>
@@ -3612,7 +3612,7 @@
       </c>
       <c r="B50" s="13" t="inlineStr">
         <is>
-          <t>Head Coach &amp; 3 Assistants</t>
+          <t>Head Coach &amp; Bench Staff</t>
         </is>
       </c>
       <c r="C50" s="13" t="inlineStr">
@@ -3629,7 +3629,7 @@
         <v>150</v>
       </c>
       <c r="F50" s="11" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="G50" s="10" t="inlineStr">
         <is>
@@ -3728,7 +3728,7 @@
         <v>105</v>
       </c>
       <c r="F56" s="11" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="G56" s="10" t="inlineStr">
         <is>
@@ -3761,7 +3761,7 @@
         <v>45</v>
       </c>
       <c r="F57" s="11" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="G57" s="10" t="inlineStr">
         <is>
@@ -4021,7 +4021,7 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>October 31, 2026</t>
+          <t>[Enter Statement Date - e.g. Oct 31, 2026]</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -4041,7 +4041,7 @@
         </is>
       </c>
       <c r="E7" s="33" t="n">
-        <v>10302.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -4086,90 +4086,90 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>Sponsorship Cheque - Gold Banner</t>
+          <t>[Deposit 1 Description]</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Oct 28, 2026</t>
+          <t>[Date]</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Local Business</t>
+          <t>[Source / Payer]</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Cheque</t>
+          <t>[Method]</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>500</v>
+        <v>0</v>
       </c>
       <c r="F11" s="10" t="inlineStr">
         <is>
-          <t>Deposited via mobile, clearing</t>
+          <t>[Pending clearance]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Late Parent Rep Fee Installment</t>
+          <t>[Deposit 2 Description]</t>
         </is>
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Oct 30, 2026</t>
+          <t>[Date]</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Parent Name</t>
+          <t>[Source / Payer]</t>
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>E-transfer</t>
+          <t>[Method]</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="F12" s="10" t="inlineStr">
         <is>
-          <t>Pending deposit acceptance</t>
+          <t>[Pending clearance]</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Bottle Drive Cash Deposit</t>
+          <t>[Deposit 3 Description]</t>
         </is>
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>Oct 31, 2026</t>
+          <t>[Date]</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>[Source / Payer]</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Cash</t>
+          <t>[Method]</t>
         </is>
       </c>
       <c r="E13" s="11" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Night deposit box</t>
+          <t>[Pending clearance]</t>
         </is>
       </c>
     </row>
@@ -4250,26 +4250,26 @@
     <row r="20">
       <c r="A20" s="13" t="inlineStr">
         <is>
-          <t>Cheque #101</t>
+          <t>[Cheque #101]</t>
         </is>
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>Oct 15, 2026</t>
+          <t>[Date]</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Amherst Minor Hockey</t>
+          <t>[Payee / Vendor]</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Tournament Entry Fee</t>
+          <t>[Description / Purpose]</t>
         </is>
       </c>
       <c r="E20" s="11" t="n">
-        <v>850</v>
+        <v>0</v>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
@@ -4280,60 +4280,60 @@
     <row r="21">
       <c r="A21" s="13" t="inlineStr">
         <is>
-          <t>Cheque #102</t>
+          <t>[Cheque #102]</t>
         </is>
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Oct 20, 2026</t>
+          <t>[Date]</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Local Print Shop</t>
+          <t>[Payee / Vendor]</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Sponsor Banner Printing</t>
+          <t>[Description / Purpose]</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>168.59</v>
+        <v>0</v>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Issued, in mail</t>
+          <t>Issued, not yet cashed</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="13" t="inlineStr">
         <is>
-          <t>Cheque #103</t>
+          <t>[Cheque #103]</t>
         </is>
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>Oct 25, 2026</t>
+          <t>[Date]</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Apparel Vendor</t>
+          <t>[Payee / Vendor]</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Practice Jerseys Deposit</t>
+          <t>[Description / Purpose]</t>
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>550</v>
+        <v>0</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>Issued</t>
+          <t>Issued, not yet cashed</t>
         </is>
       </c>
     </row>
@@ -4458,7 +4458,7 @@
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -4541,35 +4541,37 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n">
-        <v>1</v>
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>#01</t>
+        </is>
       </c>
       <c r="B5" s="10" t="inlineStr">
         <is>
-          <t>Player 1 Name</t>
+          <t>[Player 01 Legal Name]</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 1</t>
+          <t>[Parent / Guardian of Player 01]</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>parent1@example.com</t>
+          <t>[parent01@example.com]</t>
         </is>
       </c>
       <c r="E5" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F5" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G5" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H5" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I5" s="36">
         <f>SUM(E5:H5)</f>
@@ -4581,40 +4583,42 @@
       </c>
       <c r="K5" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="n">
-        <v>2</v>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>#02</t>
+        </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>Player 2 Name</t>
+          <t>[Player 02 Legal Name]</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 2</t>
+          <t>[Parent / Guardian of Player 02]</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>parent2@example.com</t>
+          <t>[parent02@example.com]</t>
         </is>
       </c>
       <c r="E6" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F6" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G6" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H6" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I6" s="36">
         <f>SUM(E6:H6)</f>
@@ -4626,40 +4630,42 @@
       </c>
       <c r="K6" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="n">
-        <v>3</v>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>#03</t>
+        </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>Player 3 Name</t>
+          <t>[Player 03 Legal Name]</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 3</t>
+          <t>[Parent / Guardian of Player 03]</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>parent3@example.com</t>
+          <t>[parent03@example.com]</t>
         </is>
       </c>
       <c r="E7" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F7" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G7" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H7" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I7" s="36">
         <f>SUM(E7:H7)</f>
@@ -4671,40 +4677,42 @@
       </c>
       <c r="K7" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="n">
-        <v>4</v>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>#04</t>
+        </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>Player 4 Name</t>
+          <t>[Player 04 Legal Name]</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 4</t>
+          <t>[Parent / Guardian of Player 04]</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>parent4@example.com</t>
+          <t>[parent04@example.com]</t>
         </is>
       </c>
       <c r="E8" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F8" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G8" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H8" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I8" s="36">
         <f>SUM(E8:H8)</f>
@@ -4716,40 +4724,42 @@
       </c>
       <c r="K8" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="n">
-        <v>5</v>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>#05</t>
+        </is>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
-          <t>Player 5 Name</t>
+          <t>[Player 05 Legal Name]</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 5</t>
+          <t>[Parent / Guardian of Player 05]</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>parent5@example.com</t>
+          <t>[parent05@example.com]</t>
         </is>
       </c>
       <c r="E9" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F9" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G9" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H9" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I9" s="36">
         <f>SUM(E9:H9)</f>
@@ -4761,40 +4771,42 @@
       </c>
       <c r="K9" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="n">
-        <v>6</v>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>#06</t>
+        </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>Player 6 Name</t>
+          <t>[Player 06 Legal Name]</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 6</t>
+          <t>[Parent / Guardian of Player 06]</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>parent6@example.com</t>
+          <t>[parent06@example.com]</t>
         </is>
       </c>
       <c r="E10" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F10" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G10" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H10" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I10" s="36">
         <f>SUM(E10:H10)</f>
@@ -4806,40 +4818,42 @@
       </c>
       <c r="K10" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n">
-        <v>7</v>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>#07</t>
+        </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t>Player 7 Name</t>
+          <t>[Player 07 Legal Name]</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 7</t>
+          <t>[Parent / Guardian of Player 07]</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>parent7@example.com</t>
+          <t>[parent07@example.com]</t>
         </is>
       </c>
       <c r="E11" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F11" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G11" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H11" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I11" s="36">
         <f>SUM(E11:H11)</f>
@@ -4851,40 +4865,42 @@
       </c>
       <c r="K11" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n">
-        <v>8</v>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>#08</t>
+        </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>Player 8 Name</t>
+          <t>[Player 08 Legal Name]</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 8</t>
+          <t>[Parent / Guardian of Player 08]</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>parent8@example.com</t>
+          <t>[parent08@example.com]</t>
         </is>
       </c>
       <c r="E12" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F12" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G12" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H12" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I12" s="36">
         <f>SUM(E12:H12)</f>
@@ -4896,40 +4912,42 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n">
-        <v>9</v>
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>#09</t>
+        </is>
       </c>
       <c r="B13" s="10" t="inlineStr">
         <is>
-          <t>Player 9 Name</t>
+          <t>[Player 09 Legal Name]</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 9</t>
+          <t>[Parent / Guardian of Player 09]</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>parent9@example.com</t>
+          <t>[parent09@example.com]</t>
         </is>
       </c>
       <c r="E13" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F13" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G13" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H13" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I13" s="36">
         <f>SUM(E13:H13)</f>
@@ -4941,40 +4959,42 @@
       </c>
       <c r="K13" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="n">
-        <v>10</v>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>#10</t>
+        </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>Player 10 Name</t>
+          <t>[Player 10 Legal Name]</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 10</t>
+          <t>[Parent / Guardian of Player 10]</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>parent10@example.com</t>
+          <t>[parent10@example.com]</t>
         </is>
       </c>
       <c r="E14" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F14" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G14" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H14" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I14" s="36">
         <f>SUM(E14:H14)</f>
@@ -4986,40 +5006,42 @@
       </c>
       <c r="K14" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="n">
-        <v>11</v>
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>#11</t>
+        </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Player 11 Name</t>
+          <t>[Player 11 Legal Name]</t>
         </is>
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 11</t>
+          <t>[Parent / Guardian of Player 11]</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>parent11@example.com</t>
+          <t>[parent11@example.com]</t>
         </is>
       </c>
       <c r="E15" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F15" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G15" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H15" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I15" s="36">
         <f>SUM(E15:H15)</f>
@@ -5031,40 +5053,42 @@
       </c>
       <c r="K15" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="n">
-        <v>12</v>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>#12</t>
+        </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Player 12 Name</t>
+          <t>[Player 12 Legal Name]</t>
         </is>
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 12</t>
+          <t>[Parent / Guardian of Player 12]</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>parent12@example.com</t>
+          <t>[parent12@example.com]</t>
         </is>
       </c>
       <c r="E16" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F16" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G16" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H16" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I16" s="36">
         <f>SUM(E16:H16)</f>
@@ -5076,40 +5100,42 @@
       </c>
       <c r="K16" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n">
-        <v>13</v>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>#13</t>
+        </is>
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Player 13 Name</t>
+          <t>[Player 13 Legal Name]</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 13</t>
+          <t>[Parent / Guardian of Player 13]</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>parent13@example.com</t>
+          <t>[parent13@example.com]</t>
         </is>
       </c>
       <c r="E17" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F17" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G17" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H17" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I17" s="36">
         <f>SUM(E17:H17)</f>
@@ -5121,40 +5147,42 @@
       </c>
       <c r="K17" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n">
-        <v>14</v>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>#14</t>
+        </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>Player 14 Name</t>
+          <t>[Player 14 Legal Name]</t>
         </is>
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 14</t>
+          <t>[Parent / Guardian of Player 14]</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>parent14@example.com</t>
+          <t>[parent14@example.com]</t>
         </is>
       </c>
       <c r="E18" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F18" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G18" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H18" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I18" s="36">
         <f>SUM(E18:H18)</f>
@@ -5166,40 +5194,42 @@
       </c>
       <c r="K18" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n">
-        <v>15</v>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>#15</t>
+        </is>
       </c>
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t>Player 15 Name</t>
+          <t>[Player 15 Legal Name]</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 15</t>
+          <t>[Parent / Guardian of Player 15]</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>parent15@example.com</t>
+          <t>[parent15@example.com]</t>
         </is>
       </c>
       <c r="E19" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F19" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G19" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H19" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I19" s="36">
         <f>SUM(E19:H19)</f>
@@ -5211,40 +5241,42 @@
       </c>
       <c r="K19" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n">
-        <v>16</v>
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>#16</t>
+        </is>
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>Player 16 Name</t>
+          <t>[Player 16 Legal Name]</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 16</t>
+          <t>[Parent / Guardian of Player 16]</t>
         </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>parent16@example.com</t>
+          <t>[parent16@example.com]</t>
         </is>
       </c>
       <c r="E20" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F20" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G20" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H20" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I20" s="36">
         <f>SUM(E20:H20)</f>
@@ -5256,40 +5288,42 @@
       </c>
       <c r="K20" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n">
-        <v>17</v>
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>#17</t>
+        </is>
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Player 17 Name</t>
+          <t>[Player 17 Legal Name]</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Parent of Player 17</t>
+          <t>[Parent / Guardian of Player 17]</t>
         </is>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>parent17@example.com</t>
+          <t>[parent17@example.com]</t>
         </is>
       </c>
       <c r="E21" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F21" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="G21" s="36" t="n">
-        <v>226.47</v>
+        <v>0</v>
       </c>
       <c r="H21" s="36" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I21" s="36">
         <f>SUM(E21:H21)</f>
@@ -5301,7 +5335,7 @@
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>Cheque on File</t>
+          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>